<commit_message>
chore: fully anonymize demo data
</commit_message>
<xml_diff>
--- a/public/CRM历史项目表-脱敏适配样表.xlsx
+++ b/public/CRM历史项目表-脱敏适配样表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-储备项目报备表（跟进中和呆滞）" sheetId="1" r:id="R7d100f9d00724e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-储备项目报备表（跟进中和呆滞）" sheetId="1" r:id="R914710a2b9254166"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -376,7 +376,7 @@
         <x:v>华东业务部</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>周岚</x:v>
+        <x:v>示例经理甲</x:v>
       </x:c>
       <x:c r="C2" s="16" t="str">
         <x:v>2026-05-10</x:v>
@@ -411,7 +411,7 @@
         <x:v>华南业务部</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>韩哲</x:v>
+        <x:v>示例经理乙</x:v>
       </x:c>
       <x:c r="C3" s="16" t="str">
         <x:v>2026-03-02</x:v>
@@ -446,7 +446,7 @@
         <x:v>华北业务部</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>叶宁</x:v>
+        <x:v>示例经理丙</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
         <x:v>2026-01-18</x:v>
@@ -481,7 +481,7 @@
         <x:v>华中业务部</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
-        <x:v>许安</x:v>
+        <x:v>示例经理丁</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
         <x:v>2026-06-03</x:v>
@@ -516,7 +516,7 @@
         <x:v>华东业务部</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>周岚</x:v>
+        <x:v>示例经理甲</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
         <x:v>2026-04-26</x:v>
@@ -551,7 +551,7 @@
         <x:v>华西业务部</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>宋敏</x:v>
+        <x:v>示例经理戊</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
         <x:v>2026-06-20</x:v>

</xml_diff>

<commit_message>
fix: complete smart import review interactions
</commit_message>
<xml_diff>
--- a/public/CRM历史项目表-脱敏适配样表.xlsx
+++ b/public/CRM历史项目表-脱敏适配样表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-储备项目报备表（跟进中和呆滞）" sheetId="1" r:id="R914710a2b9254166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-储备项目报备表（跟进中和呆滞）" sheetId="1" r:id="Redf92f992da24449"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -77,7 +78,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -119,6 +120,9 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -396,8 +400,8 @@
       <x:c r="H2" s="16" t="str">
         <x:v>跟进中</x:v>
       </x:c>
-      <x:c r="I2" s="16" t="str">
-        <x:v>71%-80%</x:v>
+      <x:c r="I2" s="19" t="n">
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="J2" s="18" t="n">
         <x:v>860</x:v>
@@ -431,8 +435,8 @@
       <x:c r="H3" s="16" t="str">
         <x:v>呆滞</x:v>
       </x:c>
-      <x:c r="I3" s="16" t="str">
-        <x:v>1%-50%</x:v>
+      <x:c r="I3" s="19" t="n">
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="J3" s="18" t="n">
         <x:v>1200</x:v>
@@ -466,7 +470,7 @@
       <x:c r="H4" s="16" t="str">
         <x:v>呆滞</x:v>
       </x:c>
-      <x:c r="I4" s="16" t="str">
+      <x:c r="I4" s="19" t="str">
         <x:v>询价类</x:v>
       </x:c>
       <x:c r="J4" s="18" t="n">
@@ -501,8 +505,8 @@
       <x:c r="H5" s="16" t="str">
         <x:v>跟进中</x:v>
       </x:c>
-      <x:c r="I5" s="16" t="str">
-        <x:v>81%-100%</x:v>
+      <x:c r="I5" s="19" t="n">
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="J5" s="18" t="n">
         <x:v>320</x:v>
@@ -536,8 +540,8 @@
       <x:c r="H6" s="16" t="str">
         <x:v>跟进中</x:v>
       </x:c>
-      <x:c r="I6" s="16" t="str">
-        <x:v>1%-50%</x:v>
+      <x:c r="I6" s="19" t="n">
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="J6" s="18" t="n">
         <x:v>1850</x:v>
@@ -571,8 +575,8 @@
       <x:c r="H7" s="16" t="str">
         <x:v>跟进中</x:v>
       </x:c>
-      <x:c r="I7" s="16" t="str">
-        <x:v>81%-100%</x:v>
+      <x:c r="I7" s="19" t="n">
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="J7" s="18" t="n">
         <x:v>240</x:v>

</xml_diff>